<commit_message>
docs: acredita HU-09 (8 pts; proyecto 141/146, 96,6 %) y actualiza backlog, estado, release plan, casos de prueba, informe de pruebas y presentacion; Excel SUS con hallazgo corregido
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/FORMATO_REGISTRO_UAT_SUS_HU09.xlsx
+++ b/docs/uat/FORMATO_REGISTRO_UAT_SUS_HU09.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1bb90464e00ae32f/Documentos/GitHub/health-access-bridge/docs/uat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="11_529C5E407BEEBE678692D6FE29274FD89D9DBADC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AA5E2C5-8384-4FF2-8A32-38388E79AF11}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="11_529C5E407BEEBE678692D6FE29274FD89D9DBADC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38072775-7C78-4425-969F-035F95C2E622}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="130">
   <si>
     <t>Health Access Bridge — Registro de la sesión de usabilidad (HU-09)</t>
   </si>
@@ -445,6 +445,12 @@
   </si>
   <si>
     <t>Pasar al backlog</t>
+  </si>
+  <si>
+    <t>#93</t>
+  </si>
+  <si>
+    <t>Corregido</t>
   </si>
 </sst>
 </file>
@@ -634,6 +640,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -642,9 +651,6 @@
     </xf>
     <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,6 +667,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1354,7 +1364,7 @@
       <c r="A3" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="30">
+      <c r="B3" s="25">
         <v>46322</v>
       </c>
       <c r="C3" s="16" t="s">
@@ -1406,7 +1416,7 @@
       <c r="A4" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="30">
+      <c r="B4" s="25">
         <v>46322</v>
       </c>
       <c r="C4" s="16" t="s">
@@ -1458,7 +1468,7 @@
       <c r="A5" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="25">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
@@ -1510,7 +1520,7 @@
       <c r="A6" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="30">
+      <c r="B6" s="25">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
@@ -1562,7 +1572,7 @@
       <c r="A7" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="30">
+      <c r="B7" s="25">
         <v>46322</v>
       </c>
       <c r="C7" s="16" t="s">
@@ -1614,7 +1624,7 @@
       <c r="A8" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="30">
+      <c r="B8" s="25">
         <v>46322</v>
       </c>
       <c r="C8" s="16" t="s">
@@ -1666,7 +1676,7 @@
       <c r="A9" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="30">
+      <c r="B9" s="25">
         <v>46322</v>
       </c>
       <c r="C9" s="16" t="s">
@@ -1718,7 +1728,7 @@
       <c r="A10" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="25">
         <v>46322</v>
       </c>
       <c r="C10" s="16" t="s">
@@ -1770,7 +1780,7 @@
       <c r="A11" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="30">
+      <c r="B11" s="25">
         <v>46322</v>
       </c>
       <c r="C11" s="16" t="s">
@@ -1822,7 +1832,7 @@
       <c r="A12" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="25">
         <v>46322</v>
       </c>
       <c r="C12" s="16" t="s">
@@ -1876,108 +1886,108 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="29">
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="30">
         <f>COUNT(O3:O12)</f>
         <v>10</v>
       </c>
-      <c r="F16" s="27"/>
+      <c r="F16" s="28"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="28">
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="29">
         <f>IF(COUNT(O3:O12)=0,"",AVERAGE(O3:O12))</f>
         <v>81.25</v>
       </c>
-      <c r="F17" s="27"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="28">
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="29">
         <f>IF(COUNT(O3:O12)=0,"",MEDIAN(O3:O12))</f>
         <v>81.25</v>
       </c>
-      <c r="F18" s="27"/>
+      <c r="F18" s="28"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="28">
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29">
         <f>IF(COUNT(O3:O12)=0,"",MIN(O3:O12))</f>
         <v>72.5</v>
       </c>
-      <c r="F19" s="27"/>
+      <c r="F19" s="28"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="28">
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="29">
         <f>IF(COUNT(O3:O12)=0,"",MAX(O3:O12))</f>
         <v>90</v>
       </c>
-      <c r="F20" s="27"/>
+      <c r="F20" s="28"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="29">
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="30">
         <f>COUNTIF(O3:O12,"&gt;=68")</f>
         <v>10</v>
       </c>
-      <c r="F21" s="27"/>
+      <c r="F21" s="28"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="28">
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29">
         <f>IFERROR(AVERAGEIFS(O3:O12,C3:C12,"Médico"),"")</f>
         <v>84</v>
       </c>
-      <c r="F22" s="27"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="28">
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="29">
         <f>IFERROR(AVERAGEIFS(O3:O12,C3:C12,"Administrador"),"")</f>
         <v>78.5</v>
       </c>
-      <c r="F23" s="27"/>
+      <c r="F23" s="28"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
@@ -3013,9 +3023,11 @@
       <c r="F3" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="G3" s="22"/>
+      <c r="G3" s="22" t="s">
+        <v>128</v>
+      </c>
       <c r="H3" s="22" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="J3" s="18" t="s">
         <v>117</v>
@@ -3044,9 +3056,11 @@
       <c r="F4" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="G4" s="22"/>
+      <c r="G4" s="22" t="s">
+        <v>128</v>
+      </c>
       <c r="H4" s="22" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>118</v>
@@ -3091,7 +3105,7 @@
       </c>
       <c r="K6" s="24">
         <f>COUNTIF(H3:H62,"Abierto")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -3110,7 +3124,7 @@
       </c>
       <c r="K7" s="24">
         <f>COUNTIF(H3:H62,"Corregido")+COUNTIF(H3:H62,"Verificado")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>